<commit_message>
Remaining work: 40-day two-stream plan (Ben 2026-10-16)
Two streams, PDF by browser print, program roll-ups after first client use, Azure with Ben at the end. Spec list waves updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/VB_スペック一覧.xlsx
+++ b/docs/VB_スペック一覧.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
@@ -748,15 +748,25 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>初回顧客利用後</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>時期未定</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B25" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>分類：Form＝画面、Batch＝一括・定期処理、Report＝集計・分析・図示・PDF、Interface＝ファイル取込・出力。サーバ内部の処理は呼び出す画面の一部としてFormに分類（一覧の備考「サーバ処理」）。</t>
         </is>
@@ -7135,7 +7145,7 @@
       </c>
       <c r="I137" s="4" t="inlineStr">
         <is>
-          <t>1f</t>
+          <t>初回顧客利用後</t>
         </is>
       </c>
       <c r="J137" s="4" t="inlineStr"/>
@@ -7181,7 +7191,7 @@
       </c>
       <c r="I138" s="4" t="inlineStr">
         <is>
-          <t>1f</t>
+          <t>初回顧客利用後</t>
         </is>
       </c>
       <c r="J138" s="4" t="inlineStr"/>
@@ -7447,7 +7457,7 @@
       </c>
       <c r="G144" s="4" t="inlineStr">
         <is>
-          <t>顧客向けレポートをPDFで出力（D-42）</t>
+          <t>顧客向けレポートをブラウザの印刷機能でPDF出力（印刷用レイアウト、追加ライブラリなし）（D-42）</t>
         </is>
       </c>
       <c r="H144" s="4" t="inlineStr">

</xml_diff>